<commit_message>
Finalized game actually done
</commit_message>
<xml_diff>
--- a/data/PropertyTycoonBoardDataTest.xlsx
+++ b/data/PropertyTycoonBoardDataTest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lewis\Documents\SoftWareEngineiering\Property_Tycoon_FX\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4694580-788B-41A7-A2E9-B69B55397778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6648AB-A4F7-43A4-B589-40EA9E3FC81E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="11295" xr2:uid="{3AB37EF7-9957-4EAE-A376-EF9CBBC9245A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3AB37EF7-9957-4EAE-A376-EF9CBBC9245A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="101">
   <si>
     <t>Go</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Pot Luck</t>
-  </si>
-  <si>
     <t>Take card</t>
   </si>
   <si>
@@ -105,9 +102,6 @@
     <t>Blue</t>
   </si>
   <si>
-    <t>Opportunity Knocks</t>
-  </si>
-  <si>
     <t>Jail/Just visiting</t>
   </si>
   <si>
@@ -171,9 +165,6 @@
     <t>Go to Jail</t>
   </si>
   <si>
-    <t>Go to jail</t>
-  </si>
-  <si>
     <t>Sirat Mews</t>
   </si>
   <si>
@@ -309,13 +300,34 @@
     <t>OppKnocks</t>
   </si>
   <si>
-    <t>Jail</t>
-  </si>
-  <si>
     <t>FreeParking</t>
   </si>
   <si>
     <t>SuperTax</t>
+  </si>
+  <si>
+    <t>Opportunity Knocks 1</t>
+  </si>
+  <si>
+    <t>Opportunity Knocks 2</t>
+  </si>
+  <si>
+    <t>Opportunity Knocks 3</t>
+  </si>
+  <si>
+    <t>Pot Luck 1</t>
+  </si>
+  <si>
+    <t>Pot Luck 2</t>
+  </si>
+  <si>
+    <t>Pot Luck 3</t>
+  </si>
+  <si>
+    <t>just visiting</t>
+  </si>
+  <si>
+    <t>Go To Jail</t>
   </si>
 </sst>
 </file>
@@ -727,7 +739,7 @@
         <v>5</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>7</v>
@@ -753,7 +765,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
@@ -762,25 +774,25 @@
         <v>3</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -812,7 +824,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s" s="0">
         <v>16</v>
@@ -847,13 +859,13 @@
         <v>3</v>
       </c>
       <c r="B7" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E7" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>19</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>14</v>
@@ -871,7 +883,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>16</v>
@@ -906,13 +918,13 @@
         <v>5</v>
       </c>
       <c r="B9" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="E9" t="s" s="0">
         <v>21</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>22</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>14</v>
@@ -930,10 +942,10 @@
         <v>6</v>
       </c>
       <c r="B10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s" s="0">
         <v>23</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>24</v>
       </c>
       <c r="F10" t="s" s="0">
         <v>17</v>
@@ -942,7 +954,7 @@
         <v>200</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -956,10 +968,10 @@
         <v>7</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F11" t="s" s="0">
         <v>17</v>
@@ -991,13 +1003,13 @@
         <v>8</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F12" t="s" s="0">
         <v>14</v>
@@ -1015,10 +1027,10 @@
         <v>9</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F13" t="s" s="0">
         <v>17</v>
@@ -1050,10 +1062,10 @@
         <v>10</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F14" t="s" s="0">
         <v>17</v>
@@ -1085,10 +1097,10 @@
         <v>11</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F15" t="s" s="0">
         <v>14</v>
@@ -1106,10 +1118,10 @@
         <v>12</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F16" t="s" s="0">
         <v>17</v>
@@ -1141,10 +1153,10 @@
         <v>13</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s" s="0">
         <v>17</v>
@@ -1153,7 +1165,7 @@
         <v>150</v>
       </c>
       <c r="I17" t="s" s="0">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
@@ -1167,10 +1179,10 @@
         <v>14</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F18" t="s" s="0">
         <v>17</v>
@@ -1202,13 +1214,13 @@
         <v>15</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H19" s="0">
         <v>160</v>
@@ -1237,10 +1249,10 @@
         <v>16</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F20" t="s" s="0">
         <v>17</v>
@@ -1249,7 +1261,7 @@
         <v>200</v>
       </c>
       <c r="I20" t="s" s="0">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
@@ -1263,10 +1275,10 @@
         <v>17</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F21" t="s" s="0">
         <v>17</v>
@@ -1298,13 +1310,13 @@
         <v>18</v>
       </c>
       <c r="B22" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E22" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="E22" t="s" s="0">
-        <v>19</v>
       </c>
       <c r="F22" t="s" s="0">
         <v>14</v>
@@ -1322,10 +1334,10 @@
         <v>19</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F23" t="s" s="0">
         <v>17</v>
@@ -1357,10 +1369,10 @@
         <v>20</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F24" t="s" s="0">
         <v>17</v>
@@ -1392,13 +1404,13 @@
         <v>21</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F25" t="s" s="0">
         <v>14</v>
@@ -1416,10 +1428,10 @@
         <v>22</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F26" t="s" s="0">
         <v>17</v>
@@ -1451,13 +1463,13 @@
         <v>23</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s" s="0">
         <v>14</v>
@@ -1475,10 +1487,10 @@
         <v>24</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s" s="0">
         <v>17</v>
@@ -1510,10 +1522,10 @@
         <v>25</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F29" t="s" s="0">
         <v>17</v>
@@ -1545,10 +1557,10 @@
         <v>26</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F30" t="s" s="0">
         <v>17</v>
@@ -1557,7 +1569,7 @@
         <v>200</v>
       </c>
       <c r="I30" t="s" s="0">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
@@ -1571,10 +1583,10 @@
         <v>27</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F31" t="s" s="0">
         <v>17</v>
@@ -1606,10 +1618,10 @@
         <v>28</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F32" t="s" s="0">
         <v>17</v>
@@ -1641,10 +1653,10 @@
         <v>29</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F33" t="s" s="0">
         <v>17</v>
@@ -1653,7 +1665,7 @@
         <v>150</v>
       </c>
       <c r="I33" t="s" s="0">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
@@ -1667,10 +1679,10 @@
         <v>30</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F34" t="s" s="0">
         <v>17</v>
@@ -1702,10 +1714,10 @@
         <v>31</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F35" t="s" s="0">
         <v>14</v>
@@ -1723,10 +1735,10 @@
         <v>32</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F36" t="s" s="0">
         <v>17</v>
@@ -1758,10 +1770,10 @@
         <v>33</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F37" t="s" s="0">
         <v>17</v>
@@ -1793,13 +1805,13 @@
         <v>34</v>
       </c>
       <c r="B38" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E38" t="s" s="0">
         <v>18</v>
-      </c>
-      <c r="D38" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="E38" t="s" s="0">
-        <v>19</v>
       </c>
       <c r="F38" t="s" s="0">
         <v>14</v>
@@ -1817,10 +1829,10 @@
         <v>35</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F39" t="s" s="0">
         <v>17</v>
@@ -1852,19 +1864,19 @@
         <v>36</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H40" s="0">
         <v>200</v>
       </c>
       <c r="I40" t="s" s="0">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
@@ -1878,10 +1890,10 @@
         <v>37</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>26</v>
+        <v>95</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F41" t="s" s="0">
         <v>14</v>
@@ -1899,10 +1911,10 @@
         <v>38</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F42" t="s" s="0">
         <v>17</v>
@@ -1934,13 +1946,13 @@
         <v>39</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F43" t="s" s="0">
         <v>14</v>
@@ -1958,10 +1970,10 @@
         <v>40</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F44" t="s" s="0">
         <v>17</v>
@@ -1990,10 +2002,10 @@
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
@@ -2001,83 +2013,83 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" t="s" s="0">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I47" s="1"/>
       <c r="J47" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" t="s" s="0">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H48" t="s" s="0">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J48" s="4">
         <v>50</v>
       </c>
       <c r="K48" t="s" s="0">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s" s="0">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H49" t="s" s="0">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J49" s="4">
         <v>100</v>
       </c>
       <c r="K49" t="s" s="0">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s" s="0">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H50" t="s" s="0">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="J50" s="4">
         <v>150</v>
       </c>
       <c r="K50" t="s" s="0">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s" s="0">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H51" t="s" s="0">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J51" s="4">
         <v>200</v>
       </c>
       <c r="K51" t="s" s="0">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s" s="0">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s" s="0">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25"/>

</xml_diff>